<commit_message>
feat: implement customer identity management, authentication services, and initial database migrations
</commit_message>
<xml_diff>
--- a/src/External/Restaurant.Persistence/Data/RestaurantData.xlsx
+++ b/src/External/Restaurant.Persistence/Data/RestaurantData.xlsx
@@ -3,14 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30219"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="55" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2B8CFCEB-DCE3-4E35-B403-3D13F320BFAD}"/>
+  <xr:revisionPtr revIDLastSave="59" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F8FBC873-156B-4098-A8FA-341F61ACB244}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="2" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Categories" sheetId="1" r:id="rId1"/>
     <sheet name="Areas" sheetId="2" r:id="rId2"/>
-    <sheet name="PersonalInfos" sheetId="3" r:id="rId3"/>
+    <sheet name="PersonalInformations" sheetId="3" r:id="rId3"/>
     <sheet name="Images" sheetId="4" r:id="rId4"/>
     <sheet name="Roles" sheetId="5" r:id="rId5"/>
     <sheet name="Products" sheetId="6" r:id="rId6"/>
@@ -952,58 +952,58 @@
     <t>IsActive</t>
   </si>
   <si>
+    <t>RoleId</t>
+  </si>
+  <si>
+    <t>660e8400-e29b-41d4-a716-446655440001</t>
+  </si>
+  <si>
+    <t>nguyenvana</t>
+  </si>
+  <si>
+    <t>nguyenvana@restaurant.com</t>
+  </si>
+  <si>
+    <t>660e8400-e29b-41d4-a716-446655440002</t>
+  </si>
+  <si>
+    <t>tranthib</t>
+  </si>
+  <si>
+    <t>tranthib@restaurant.com</t>
+  </si>
+  <si>
+    <t>660e8400-e29b-41d4-a716-446655440003</t>
+  </si>
+  <si>
+    <t>phamvanc</t>
+  </si>
+  <si>
+    <t>phamvanc@restaurant.com</t>
+  </si>
+  <si>
+    <t>660e8400-e29b-41d4-a716-446655440004</t>
+  </si>
+  <si>
+    <t>hoangthid</t>
+  </si>
+  <si>
+    <t>hoangthid@restaurant.com</t>
+  </si>
+  <si>
+    <t>660e8400-e29b-41d4-a716-446655440005</t>
+  </si>
+  <si>
+    <t>vuvane</t>
+  </si>
+  <si>
+    <t>vuvane@restaurant.com</t>
+  </si>
+  <si>
+    <t>UserId</t>
+  </si>
+  <si>
     <t>PIId</t>
-  </si>
-  <si>
-    <t>RoleId</t>
-  </si>
-  <si>
-    <t>660e8400-e29b-41d4-a716-446655440001</t>
-  </si>
-  <si>
-    <t>nguyenvana</t>
-  </si>
-  <si>
-    <t>nguyenvana@restaurant.com</t>
-  </si>
-  <si>
-    <t>660e8400-e29b-41d4-a716-446655440002</t>
-  </si>
-  <si>
-    <t>tranthib</t>
-  </si>
-  <si>
-    <t>tranthib@restaurant.com</t>
-  </si>
-  <si>
-    <t>660e8400-e29b-41d4-a716-446655440003</t>
-  </si>
-  <si>
-    <t>phamvanc</t>
-  </si>
-  <si>
-    <t>phamvanc@restaurant.com</t>
-  </si>
-  <si>
-    <t>660e8400-e29b-41d4-a716-446655440004</t>
-  </si>
-  <si>
-    <t>hoangthid</t>
-  </si>
-  <si>
-    <t>hoangthid@restaurant.com</t>
-  </si>
-  <si>
-    <t>660e8400-e29b-41d4-a716-446655440005</t>
-  </si>
-  <si>
-    <t>vuvane</t>
-  </si>
-  <si>
-    <t>vuvane@restaurant.com</t>
-  </si>
-  <si>
-    <t>UserId</t>
   </si>
   <si>
     <t>770e8400-e29b-41d4-a716-446655440001</t>
@@ -1577,55 +1577,73 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF8FEB0D-1DD7-4FB2-BE63-A7B82FDC9377}">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>318</v>
+      </c>
+      <c r="C1" t="s">
         <v>319</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:3">
       <c r="A2" s="1" t="s">
         <v>320</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
+        <v>303</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
       <c r="A3" s="1" t="s">
         <v>321</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2">
+        <v>306</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
       <c r="A4" s="1" t="s">
         <v>322</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2">
+        <v>309</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
       <c r="A5" s="1" t="s">
         <v>323</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2">
+        <v>312</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
       <c r="A6" s="1" t="s">
         <v>324</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>316</v>
+        <v>315</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -2240,6 +2258,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F21E56BB-69E4-4B40-AA01-C2AC06882E04}">
   <dimension ref="A1:J6"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="4" max="4" width="10.140625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
@@ -4524,10 +4545,10 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1CCD539-6B21-4873-B496-653E1A3CFE0A}">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:6">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4546,19 +4567,16 @@
       <c r="F1" t="s">
         <v>302</v>
       </c>
-      <c r="G1" t="s">
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="1" t="s">
         <v>303</v>
       </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" s="1" t="s">
+      <c r="B2" t="s">
         <v>304</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>305</v>
-      </c>
-      <c r="C2" t="s">
-        <v>306</v>
       </c>
       <c r="D2">
         <v>674000</v>
@@ -4566,22 +4584,19 @@
       <c r="E2" t="b">
         <v>1</v>
       </c>
-      <c r="F2" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="G2" t="s">
+      <c r="F2" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:6">
       <c r="A3" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="B3" t="s">
         <v>307</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>308</v>
-      </c>
-      <c r="C3" t="s">
-        <v>309</v>
       </c>
       <c r="D3">
         <v>669620</v>
@@ -4589,22 +4604,19 @@
       <c r="E3" t="b">
         <v>1</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="G3" t="s">
+      <c r="F3" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:6">
       <c r="A4" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="B4" t="s">
         <v>310</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>311</v>
-      </c>
-      <c r="C4" t="s">
-        <v>312</v>
       </c>
       <c r="D4">
         <v>684796</v>
@@ -4612,22 +4624,19 @@
       <c r="E4" t="b">
         <v>1</v>
       </c>
-      <c r="F4" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="G4" t="s">
+      <c r="F4" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:6">
       <c r="A5" s="1" t="s">
+        <v>312</v>
+      </c>
+      <c r="B5" t="s">
         <v>313</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>314</v>
-      </c>
-      <c r="C5" t="s">
-        <v>315</v>
       </c>
       <c r="D5">
         <v>988054</v>
@@ -4635,22 +4644,19 @@
       <c r="E5" t="b">
         <v>1</v>
       </c>
-      <c r="F5" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="G5" t="s">
+      <c r="F5" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:6">
       <c r="A6" s="1" t="s">
+        <v>315</v>
+      </c>
+      <c r="B6" t="s">
         <v>316</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>317</v>
-      </c>
-      <c r="C6" t="s">
-        <v>318</v>
       </c>
       <c r="D6">
         <v>802864</v>
@@ -4658,10 +4664,7 @@
       <c r="E6" t="b">
         <v>1</v>
       </c>
-      <c r="F6" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="G6" t="s">
+      <c r="F6" t="s">
         <v>169</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add Type column to Area entity and update PIId relation in Customer model
</commit_message>
<xml_diff>
--- a/src/External/Restaurant.Persistence/Data/RestaurantData.xlsx
+++ b/src/External/Restaurant.Persistence/Data/RestaurantData.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30219"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="59" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F8FBC873-156B-4098-A8FA-341F61ACB244}"/>
+  <xr:revisionPtr revIDLastSave="69" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17ED05FC-D835-4661-9EAC-ED6A10D4CBC5}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="2" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="8" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Categories" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="641" uniqueCount="357">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="645" uniqueCount="361">
   <si>
     <t>Id</t>
   </si>
@@ -118,6 +118,9 @@
     <t>Side Dishes</t>
   </si>
   <si>
+    <t>Type</t>
+  </si>
+  <si>
     <t>Status</t>
   </si>
   <si>
@@ -130,6 +133,9 @@
     <t>The primary dining area on the ground floor.</t>
   </si>
   <si>
+    <t>Standard</t>
+  </si>
+  <si>
     <t>Active</t>
   </si>
   <si>
@@ -142,6 +148,9 @@
     <t>Outdoor seating area with heating.</t>
   </si>
   <si>
+    <t>Outdoor</t>
+  </si>
+  <si>
     <t>D3F2C2C6-AE79-453D-9F31-B2C3A8D4D6B5</t>
   </si>
   <si>
@@ -149,6 +158,9 @@
   </si>
   <si>
     <t>Exclusive private dining room on the second floor.</t>
+  </si>
+  <si>
+    <t>VIP</t>
   </si>
   <si>
     <t>FirstName</t>
@@ -1167,7 +1179,134 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="7">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Consolas"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1178,6 +1317,20 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3137F4F4-FD0C-4D2F-B811-820191D5994F}" name="Table1" displayName="Table1" ref="A1:E4" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
+  <autoFilter ref="A1:E4" xr:uid="{3137F4F4-FD0C-4D2F-B811-820191D5994F}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{246F2EF2-2C35-4991-9BC4-D9B3E8DFE192}" name="Id" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{021D5693-D9EC-4A49-BFD1-A1763F1415B5}" name="Name" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{E360800A-C5F3-445E-82B9-2CEE0D3CF920}" name="Description" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{4394E3CD-6D41-427F-9E64-36A2975D6526}" name="Type" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{9FF92C23-B8B0-4E0E-BAC4-B32450B684D7}" name="Status" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1585,65 +1738,65 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>318</v>
+        <v>322</v>
       </c>
       <c r="C1" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="1" t="s">
-        <v>320</v>
+        <v>324</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="1" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>306</v>
+        <v>310</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="1" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="1" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="1" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>
@@ -1661,27 +1814,27 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="C1" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="D1" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="E1" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="B2" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="C2" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="D2" t="b">
         <v>1</v>
@@ -1692,13 +1845,13 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="B3" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="C3" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="D3" t="b">
         <v>1</v>
@@ -1709,13 +1862,13 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
       <c r="B4" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="C4" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="D4" t="b">
         <v>1</v>
@@ -1726,13 +1879,13 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="B5" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="C5" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="D5" t="b">
         <v>1</v>
@@ -1743,13 +1896,13 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>331</v>
+        <v>335</v>
       </c>
       <c r="B6" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="C6" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D6" t="b">
         <v>1</v>
@@ -1760,13 +1913,13 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="B7" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="C7" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="D7" t="b">
         <v>1</v>
@@ -1777,13 +1930,13 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>333</v>
+        <v>337</v>
       </c>
       <c r="B8" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="C8" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="D8" t="b">
         <v>1</v>
@@ -1794,13 +1947,13 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>334</v>
+        <v>338</v>
       </c>
       <c r="B9" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="C9" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="D9" t="b">
         <v>1</v>
@@ -1811,13 +1964,13 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="B10" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="C10" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="D10" t="b">
         <v>1</v>
@@ -1828,13 +1981,13 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>336</v>
+        <v>340</v>
       </c>
       <c r="B11" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="C11" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="D11" t="b">
         <v>1</v>
@@ -1845,13 +1998,13 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
       <c r="B12" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="C12" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="D12" t="b">
         <v>1</v>
@@ -1862,13 +2015,13 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="B13" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="C13" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="D13" t="b">
         <v>1</v>
@@ -1879,13 +2032,13 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="B14" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="C14" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D14" t="b">
         <v>1</v>
@@ -1896,13 +2049,13 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="B15" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="C15" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="D15" t="b">
         <v>1</v>
@@ -1913,13 +2066,13 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="B16" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="C16" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D16" t="b">
         <v>1</v>
@@ -1930,13 +2083,13 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="B17" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="C17" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="D17" t="b">
         <v>1</v>
@@ -1947,13 +2100,13 @@
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
       <c r="B18" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="C18" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="D18" t="b">
         <v>1</v>
@@ -1964,13 +2117,13 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
       <c r="B19" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="C19" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="D19" t="b">
         <v>1</v>
@@ -1981,13 +2134,13 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="B20" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="C20" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="D20" t="b">
         <v>1</v>
@@ -1998,13 +2151,13 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="B21" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="C21" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="D21" t="b">
         <v>1</v>
@@ -2015,13 +2168,13 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
       <c r="B22" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="C22" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="D22" t="b">
         <v>1</v>
@@ -2032,13 +2185,13 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="B23" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="C23" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="D23" t="b">
         <v>1</v>
@@ -2049,13 +2202,13 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
       <c r="B24" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="C24" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="D24" t="b">
         <v>1</v>
@@ -2066,13 +2219,13 @@
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>350</v>
+        <v>354</v>
       </c>
       <c r="B25" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="C25" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="D25" t="b">
         <v>1</v>
@@ -2083,13 +2236,13 @@
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>351</v>
+        <v>355</v>
       </c>
       <c r="B26" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="C26" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="D26" t="b">
         <v>1</v>
@@ -2100,13 +2253,13 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="B27" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="C27" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="D27" t="b">
         <v>1</v>
@@ -2117,13 +2270,13 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="B28" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="C28" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="D28" t="b">
         <v>1</v>
@@ -2134,13 +2287,13 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="B29" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="C29" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="D29" t="b">
         <v>1</v>
@@ -2151,13 +2304,13 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
       <c r="B30" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="C30" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="D30" t="b">
         <v>1</v>
@@ -2168,13 +2321,13 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
       <c r="B31" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="C31" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="D31" t="b">
         <v>1</v>
@@ -2190,10 +2343,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A69DCA73-68AB-4489-A60C-ADBBB6F14399}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="43.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="44.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="44.42578125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:5">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2206,51 +2365,66 @@
       <c r="D1" s="3" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="2" spans="1:4">
+      <c r="E1" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
       <c r="A2" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
+        <v>29</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
       <c r="A3" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
+    </row>
+    <row r="4" spans="1:5">
       <c r="A4" s="2" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>28</v>
+        <v>38</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -2267,42 +2441,42 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="C1" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="D1" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="E1" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="F1" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="G1" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="H1" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="I1" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="J1" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" s="1" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="C2" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="D2" s="4">
         <v>33008</v>
@@ -2311,13 +2485,13 @@
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="G2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="H2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="I2">
         <v>901234567</v>
@@ -2328,13 +2502,13 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" s="1" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B3" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C3" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D3" s="4">
         <v>33838</v>
@@ -2343,13 +2517,13 @@
         <v>0</v>
       </c>
       <c r="F3" t="s">
+        <v>57</v>
+      </c>
+      <c r="G3" t="s">
+        <v>58</v>
+      </c>
+      <c r="H3" t="s">
         <v>53</v>
-      </c>
-      <c r="G3" t="s">
-        <v>54</v>
-      </c>
-      <c r="H3" t="s">
-        <v>49</v>
       </c>
       <c r="I3">
         <v>912345678</v>
@@ -2360,13 +2534,13 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" s="1" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B4" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C4" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="D4" s="4">
         <v>34768</v>
@@ -2375,13 +2549,13 @@
         <v>1</v>
       </c>
       <c r="F4" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="G4" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="H4" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="I4">
         <v>923456789</v>
@@ -2392,13 +2566,13 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="1" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B5" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="C5" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="D5" s="4">
         <v>36104</v>
@@ -2407,13 +2581,13 @@
         <v>0</v>
       </c>
       <c r="F5" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="G5" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="H5" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="I5">
         <v>934567890</v>
@@ -2424,13 +2598,13 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" s="1" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="B6" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C6" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="D6" s="4">
         <v>32344</v>
@@ -2439,13 +2613,13 @@
         <v>1</v>
       </c>
       <c r="F6" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="G6" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="H6" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="I6">
         <v>945678901</v>
@@ -2469,33 +2643,33 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C1" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="D1" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="E1" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="F1" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="G1" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="B2" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C2" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D2" t="b">
         <v>1</v>
@@ -2504,21 +2678,21 @@
         <v>328.74</v>
       </c>
       <c r="F2" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="G2" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B3" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C3" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D3" t="b">
         <v>1</v>
@@ -2527,21 +2701,21 @@
         <v>9.76</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="B4" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="C4" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D4" t="b">
         <v>1</v>
@@ -2550,21 +2724,21 @@
         <v>239.33</v>
       </c>
       <c r="F4" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="G4" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="B5" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="C5" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D5" t="b">
         <v>1</v>
@@ -2573,21 +2747,21 @@
         <v>181.91</v>
       </c>
       <c r="F5" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="G5" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B6" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="C6" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D6" t="b">
         <v>1</v>
@@ -2596,21 +2770,21 @@
         <v>96.88</v>
       </c>
       <c r="F6" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="G6" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B7" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="C7" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D7" t="b">
         <v>1</v>
@@ -2619,21 +2793,21 @@
         <v>33.75</v>
       </c>
       <c r="F7" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="G7" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B8" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="C8" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D8" t="b">
         <v>1</v>
@@ -2642,21 +2816,21 @@
         <v>161.56</v>
       </c>
       <c r="F8" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="G8" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B9" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C9" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D9" t="b">
         <v>1</v>
@@ -2665,21 +2839,21 @@
         <v>50.77</v>
       </c>
       <c r="F9" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="G9" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="B10" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D10" t="b">
         <v>1</v>
@@ -2688,21 +2862,21 @@
         <v>65.02</v>
       </c>
       <c r="F10" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="G10" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B11" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C11" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D11" t="b">
         <v>1</v>
@@ -2711,21 +2885,21 @@
         <v>124.85</v>
       </c>
       <c r="F11" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="G11" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="B12" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="C12" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D12" t="b">
         <v>1</v>
@@ -2734,21 +2908,21 @@
         <v>97.29</v>
       </c>
       <c r="F12" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="G12" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="B13" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="C13" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D13" t="b">
         <v>1</v>
@@ -2757,21 +2931,21 @@
         <v>127.72</v>
       </c>
       <c r="F13" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="G13" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="B14" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="C14" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="D14" t="b">
         <v>1</v>
@@ -2780,21 +2954,21 @@
         <v>47.86</v>
       </c>
       <c r="F14" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="G14" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="B15" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="C15" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D15" t="b">
         <v>1</v>
@@ -2803,21 +2977,21 @@
         <v>11.46</v>
       </c>
       <c r="F15" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="G15" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="B16" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="C16" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D16" t="b">
         <v>1</v>
@@ -2826,21 +3000,21 @@
         <v>91.76</v>
       </c>
       <c r="F16" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G16" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="B17" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="C17" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D17" t="b">
         <v>1</v>
@@ -2849,21 +3023,21 @@
         <v>157.78</v>
       </c>
       <c r="F17" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="G17" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B18" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="C18" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="D18" t="b">
         <v>1</v>
@@ -2872,21 +3046,21 @@
         <v>26.03</v>
       </c>
       <c r="F18" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="G18" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
     </row>
     <row r="19" spans="1:7">
       <c r="A19" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B19" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C19" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D19" t="b">
         <v>1</v>
@@ -2895,21 +3069,21 @@
         <v>20.29</v>
       </c>
       <c r="F19" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="G19" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
     </row>
     <row r="20" spans="1:7">
       <c r="A20" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="B20" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="C20" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D20" t="b">
         <v>1</v>
@@ -2918,21 +3092,21 @@
         <v>8.6300000000000008</v>
       </c>
       <c r="F20" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="G20" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="B21" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="C21" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D21" t="b">
         <v>1</v>
@@ -2941,21 +3115,21 @@
         <v>60.75</v>
       </c>
       <c r="F21" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="G21" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
     </row>
     <row r="22" spans="1:7">
       <c r="A22" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B22" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C22" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D22" t="b">
         <v>1</v>
@@ -2964,21 +3138,21 @@
         <v>454.65</v>
       </c>
       <c r="F22" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="G22" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
     </row>
     <row r="23" spans="1:7">
       <c r="A23" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="B23" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="C23" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D23" t="b">
         <v>1</v>
@@ -2987,21 +3161,21 @@
         <v>135.88</v>
       </c>
       <c r="F23" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="G23" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
     </row>
     <row r="24" spans="1:7">
       <c r="A24" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="B24" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="C24" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D24" t="b">
         <v>1</v>
@@ -3010,21 +3184,21 @@
         <v>255.67</v>
       </c>
       <c r="F24" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="G24" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
     </row>
     <row r="25" spans="1:7">
       <c r="A25" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="B25" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="C25" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D25" t="b">
         <v>1</v>
@@ -3033,21 +3207,21 @@
         <v>81.92</v>
       </c>
       <c r="F25" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="G25" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
     </row>
     <row r="26" spans="1:7">
       <c r="A26" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="B26" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="C26" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D26" t="b">
         <v>1</v>
@@ -3056,21 +3230,21 @@
         <v>288.77999999999997</v>
       </c>
       <c r="F26" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="G26" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
     </row>
     <row r="27" spans="1:7">
       <c r="A27" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="B27" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="C27" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D27" t="b">
         <v>1</v>
@@ -3079,21 +3253,21 @@
         <v>49.91</v>
       </c>
       <c r="F27" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="G27" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
     </row>
     <row r="28" spans="1:7">
       <c r="A28" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="B28" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="C28" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D28" t="b">
         <v>1</v>
@@ -3102,21 +3276,21 @@
         <v>108.12</v>
       </c>
       <c r="F28" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="G28" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
     </row>
     <row r="29" spans="1:7">
       <c r="A29" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="B29" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="C29" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D29" t="b">
         <v>1</v>
@@ -3125,21 +3299,21 @@
         <v>102.67</v>
       </c>
       <c r="F29" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="G29" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
     </row>
     <row r="30" spans="1:7">
       <c r="A30" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="B30" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="C30" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D30" t="b">
         <v>1</v>
@@ -3148,21 +3322,21 @@
         <v>203.67</v>
       </c>
       <c r="F30" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="G30" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
     </row>
     <row r="31" spans="1:7">
       <c r="A31" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="B31" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="C31" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D31" t="b">
         <v>1</v>
@@ -3171,10 +3345,10 @@
         <v>53.44</v>
       </c>
       <c r="F31" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="G31" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
     </row>
   </sheetData>
@@ -3200,46 +3374,46 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="B2" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="C2" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="B3" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="C3" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="B4" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="C4" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="B5" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="C5" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
     </row>
   </sheetData>
@@ -3263,24 +3437,24 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="E1" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="F1" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="B2" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C2" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="D2" t="b">
         <v>1</v>
@@ -3294,13 +3468,13 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="B3" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C3" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="D3" t="b">
         <v>1</v>
@@ -3314,13 +3488,13 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="B4" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="C4" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="D4" t="b">
         <v>1</v>
@@ -3334,13 +3508,13 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="B5" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="C5" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="D5" t="b">
         <v>1</v>
@@ -3354,13 +3528,13 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="B6" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="C6" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="D6" t="b">
         <v>1</v>
@@ -3374,13 +3548,13 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="B7" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="C7" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="D7" t="b">
         <v>1</v>
@@ -3394,13 +3568,13 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="B8" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="C8" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="D8" t="b">
         <v>1</v>
@@ -3414,13 +3588,13 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="B9" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C9" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="D9" t="b">
         <v>1</v>
@@ -3434,13 +3608,13 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="B10" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C10" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="D10" t="b">
         <v>1</v>
@@ -3454,13 +3628,13 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="B11" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C11" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="D11" t="b">
         <v>1</v>
@@ -3474,13 +3648,13 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="B12" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="C12" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="D12" t="b">
         <v>1</v>
@@ -3494,13 +3668,13 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="B13" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="C13" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="D13" t="b">
         <v>1</v>
@@ -3514,13 +3688,13 @@
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="B14" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="C14" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="D14" t="b">
         <v>1</v>
@@ -3534,13 +3708,13 @@
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="B15" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="C15" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="D15" t="b">
         <v>1</v>
@@ -3554,13 +3728,13 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="B16" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="C16" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="D16" t="b">
         <v>1</v>
@@ -3574,13 +3748,13 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="B17" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="C17" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="D17" t="b">
         <v>1</v>
@@ -3594,13 +3768,13 @@
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="B18" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="C18" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="D18" t="b">
         <v>1</v>
@@ -3614,13 +3788,13 @@
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="B19" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C19" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="D19" t="b">
         <v>1</v>
@@ -3634,13 +3808,13 @@
     </row>
     <row r="20" spans="1:6">
       <c r="A20" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="B20" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="C20" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="D20" t="b">
         <v>1</v>
@@ -3654,13 +3828,13 @@
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="B21" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="C21" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="D21" t="b">
         <v>1</v>
@@ -3674,13 +3848,13 @@
     </row>
     <row r="22" spans="1:6">
       <c r="A22" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="B22" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C22" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="D22" t="b">
         <v>1</v>
@@ -3694,13 +3868,13 @@
     </row>
     <row r="23" spans="1:6">
       <c r="A23" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="B23" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="C23" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="D23" t="b">
         <v>1</v>
@@ -3714,13 +3888,13 @@
     </row>
     <row r="24" spans="1:6">
       <c r="A24" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="B24" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="C24" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="D24" t="b">
         <v>1</v>
@@ -3734,13 +3908,13 @@
     </row>
     <row r="25" spans="1:6">
       <c r="A25" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="B25" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="C25" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="D25" t="b">
         <v>1</v>
@@ -3754,13 +3928,13 @@
     </row>
     <row r="26" spans="1:6">
       <c r="A26" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="B26" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="C26" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="D26" t="b">
         <v>1</v>
@@ -3774,13 +3948,13 @@
     </row>
     <row r="27" spans="1:6">
       <c r="A27" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="B27" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="C27" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="D27" t="b">
         <v>1</v>
@@ -3794,13 +3968,13 @@
     </row>
     <row r="28" spans="1:6">
       <c r="A28" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="B28" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="C28" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="D28" t="b">
         <v>1</v>
@@ -3814,13 +3988,13 @@
     </row>
     <row r="29" spans="1:6">
       <c r="A29" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="B29" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="C29" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="D29" t="b">
         <v>1</v>
@@ -3834,13 +4008,13 @@
     </row>
     <row r="30" spans="1:6">
       <c r="A30" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="B30" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="C30" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="D30" t="b">
         <v>1</v>
@@ -3854,13 +4028,13 @@
     </row>
     <row r="31" spans="1:6">
       <c r="A31" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="B31" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="C31" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="D31" t="b">
         <v>1</v>
@@ -3887,30 +4061,30 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="C1" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="D1" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="E1" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="B2" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="C2">
         <v>65000</v>
       </c>
       <c r="D2" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -3918,16 +4092,16 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="B3" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="C3">
         <v>55000</v>
       </c>
       <c r="D3" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -3935,16 +4109,16 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="B4" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="C4">
         <v>60000</v>
       </c>
       <c r="D4" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -3952,16 +4126,16 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="B5" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="C5">
         <v>55000</v>
       </c>
       <c r="D5" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -3969,16 +4143,16 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="B6" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="C6">
         <v>55000</v>
       </c>
       <c r="D6" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -3986,16 +4160,16 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="B7" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="C7">
         <v>75000</v>
       </c>
       <c r="D7" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="E7">
         <v>0</v>
@@ -4003,16 +4177,16 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="B8" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="C8">
         <v>95000</v>
       </c>
       <c r="D8" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="E8">
         <v>0</v>
@@ -4020,16 +4194,16 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="B9" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="C9">
         <v>120000</v>
       </c>
       <c r="D9" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="E9">
         <v>0</v>
@@ -4037,16 +4211,16 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="B10" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="C10">
         <v>85000</v>
       </c>
       <c r="D10" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="E10">
         <v>0</v>
@@ -4054,16 +4228,16 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="B11" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="C11">
         <v>80000</v>
       </c>
       <c r="D11" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="E11">
         <v>0</v>
@@ -4071,16 +4245,16 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="B12" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="C12">
         <v>45000</v>
       </c>
       <c r="D12" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="E12">
         <v>120</v>
@@ -4088,16 +4262,16 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="B13" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="C13">
         <v>40000</v>
       </c>
       <c r="D13" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="E13">
         <v>0</v>
@@ -4105,16 +4279,16 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="B14" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="C14">
         <v>35000</v>
       </c>
       <c r="D14" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="E14">
         <v>0</v>
@@ -4122,16 +4296,16 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="B15" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="C15">
         <v>55000</v>
       </c>
       <c r="D15" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="E15">
         <v>0</v>
@@ -4139,16 +4313,16 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="B16" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="C16">
         <v>25000</v>
       </c>
       <c r="D16" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="E16">
         <v>0</v>
@@ -4156,16 +4330,16 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="B17" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="C17">
         <v>45000</v>
       </c>
       <c r="D17" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="E17">
         <v>0</v>
@@ -4173,16 +4347,16 @@
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="B18" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="C18">
         <v>40000</v>
       </c>
       <c r="D18" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="E18">
         <v>0</v>
@@ -4190,16 +4364,16 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="B19" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="C19">
         <v>35000</v>
       </c>
       <c r="D19" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="E19">
         <v>0</v>
@@ -4207,16 +4381,16 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="B20" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="C20">
         <v>30000</v>
       </c>
       <c r="D20" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="E20">
         <v>0</v>
@@ -4224,16 +4398,16 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="B21" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="C21">
         <v>25000</v>
       </c>
       <c r="D21" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="E21">
         <v>0</v>
@@ -4241,16 +4415,16 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="B22" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="C22">
         <v>30000</v>
       </c>
       <c r="D22" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="E22">
         <v>500</v>
@@ -4258,16 +4432,16 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="B23" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="C23">
         <v>32000</v>
       </c>
       <c r="D23" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="E23">
         <v>500</v>
@@ -4275,16 +4449,16 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="B24" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="C24">
         <v>150000</v>
       </c>
       <c r="D24" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="E24">
         <v>50</v>
@@ -4292,16 +4466,16 @@
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="B25" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="C25">
         <v>30000</v>
       </c>
       <c r="D25" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="E25">
         <v>120</v>
@@ -4309,16 +4483,16 @@
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="B26" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="C26">
         <v>40000</v>
       </c>
       <c r="D26" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="E26">
         <v>0</v>
@@ -4326,16 +4500,16 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="B27" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="C27">
         <v>35000</v>
       </c>
       <c r="D27" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="E27">
         <v>0</v>
@@ -4343,16 +4517,16 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="B28" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="C28">
         <v>20000</v>
       </c>
       <c r="D28" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="E28">
         <v>200</v>
@@ -4360,16 +4534,16 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="B29" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="C29">
         <v>35000</v>
       </c>
       <c r="D29" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="E29">
         <v>0</v>
@@ -4377,16 +4551,16 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="B30" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="C30">
         <v>40000</v>
       </c>
       <c r="D30" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="E30">
         <v>0</v>
@@ -4394,16 +4568,16 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="B31" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="C31">
         <v>45000</v>
       </c>
       <c r="D31" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="E31">
         <v>0</v>
@@ -4424,118 +4598,118 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="C1" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="D1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E1" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="B2" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="C2">
         <v>2</v>
       </c>
       <c r="D2" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="E2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="B3" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="C3">
         <v>4</v>
       </c>
       <c r="D3" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="E3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="B4" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="C4">
         <v>4</v>
       </c>
       <c r="D4" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="E4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="B5" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="C5">
         <v>2</v>
       </c>
       <c r="D5" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="E5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="1" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="B6" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="C6">
         <v>4</v>
       </c>
       <c r="D6" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="E6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>296</v>
+        <v>300</v>
       </c>
       <c r="B7" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
       <c r="C7">
         <v>8</v>
       </c>
       <c r="D7" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="E7" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -4553,30 +4727,30 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="C1" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="D1" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="E1" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="F1" t="s">
-        <v>302</v>
+        <v>306</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="1" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="B2" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="C2" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="D2">
         <v>674000</v>
@@ -4585,18 +4759,18 @@
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="1" t="s">
-        <v>306</v>
+        <v>310</v>
       </c>
       <c r="B3" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="C3" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
       <c r="D3">
         <v>669620</v>
@@ -4605,18 +4779,18 @@
         <v>1</v>
       </c>
       <c r="F3" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="1" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="B4" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="C4" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
       <c r="D4">
         <v>684796</v>
@@ -4625,18 +4799,18 @@
         <v>1</v>
       </c>
       <c r="F4" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="1" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="B5" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="C5" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
       <c r="D5">
         <v>988054</v>
@@ -4645,18 +4819,18 @@
         <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="1" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
       <c r="B6" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="C6" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
       <c r="D6">
         <v>802864</v>
@@ -4665,7 +4839,7 @@
         <v>1</v>
       </c>
       <c r="F6" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
     </row>
   </sheetData>

</xml_diff>